<commit_message>
competition audit json completed
</commit_message>
<xml_diff>
--- a/briefs/Creative brief_01_harry-nikki-mansoor.xlsx
+++ b/briefs/Creative brief_01_harry-nikki-mansoor.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Ramakant\VSCode-projects\delicut-creative-workflow\briefs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D31B8F88-E070-4C42-92BD-A8C5EFB93E4C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{21F32B29-67DC-4369-95C9-737F72CBD235}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="43">
   <si>
     <t>Persona</t>
   </si>
@@ -116,6 +116,40 @@
   </si>
   <si>
     <t>Diabetes meal plan</t>
+  </si>
+  <si>
+    <t>Reasons to buy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">trust (4.7 stars on google reviews); accurate calorie count; </t>
+  </si>
+  <si>
+    <t>delicious chef-prepared meals; frictionless delivery experience</t>
+  </si>
+  <si>
+    <t>certified by nutritionists; customised for diabetic patients</t>
+  </si>
+  <si>
+    <t xml:space="preserve">41-year-old UAE resident, female, suffering with Polycystic Ovary Syndrome; </t>
+  </si>
+  <si>
+    <t>needs food to help reducing inflammation and managing insulin levels through high-fiber, low-glycemic, and whole foods</t>
+  </si>
+  <si>
+    <t>PCOS friendly diet that foucses on balance, steady blood sugar, balanced meals &amp; nutrients to manage hormones</t>
+  </si>
+  <si>
+    <t>PCOS Meal Plan</t>
+  </si>
+  <si>
+    <t>Goal-critical snacks to reduce crashes and support hormonal balance
+Less decision fatigue → better consistency</t>
+  </si>
+  <si>
+    <t>show customers with tired expressions, mid-day slumps, mirror checks, skipped workouts, never medical or clinical.</t>
+  </si>
+  <si>
+    <t>cheaper than takeout; pause anytime; big on taste; global cuisine</t>
   </si>
 </sst>
 </file>
@@ -392,13 +426,14 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:F997"/>
+  <dimension ref="A1:G997"/>
   <sheetFormatPr defaultColWidth="12.6640625" defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="6" width="27.6640625" customWidth="1"/>
+    <col min="7" max="7" width="25.44140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="1"/>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -406,7 +441,7 @@
       <c r="E1" s="1"/>
       <c r="F1" s="1"/>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="1"/>
       <c r="B2" s="1"/>
       <c r="C2" s="1"/>
@@ -414,7 +449,7 @@
       <c r="E2" s="1"/>
       <c r="F2" s="1"/>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:7" ht="26.4" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>0</v>
       </c>
@@ -433,8 +468,11 @@
       <c r="F3" s="2" t="s">
         <v>29</v>
       </c>
-    </row>
-    <row r="4" spans="1:6" ht="52.8" x14ac:dyDescent="0.25">
+      <c r="G3" s="2" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" ht="52.8" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
         <v>5</v>
       </c>
@@ -453,8 +491,11 @@
       <c r="F4" s="3" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="5" spans="1:6" ht="52.8" x14ac:dyDescent="0.25">
+      <c r="G4" s="3" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" ht="52.8" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
         <v>10</v>
       </c>
@@ -473,8 +514,11 @@
       <c r="F5" s="3" t="s">
         <v>30</v>
       </c>
-    </row>
-    <row r="6" spans="1:6" ht="52.8" x14ac:dyDescent="0.25">
+      <c r="G5" s="3" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" ht="52.8" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
         <v>14</v>
       </c>
@@ -493,8 +537,11 @@
       <c r="F6" s="3" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="7" spans="1:6" ht="52.8" x14ac:dyDescent="0.25">
+      <c r="G6" s="3" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" ht="52.8" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
         <v>19</v>
       </c>
@@ -513,8 +560,11 @@
       <c r="F7" s="3" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="8" spans="1:6" ht="52.8" x14ac:dyDescent="0.25">
+      <c r="G7" s="3" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" ht="52.8" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
         <v>24</v>
       </c>
@@ -533,16 +583,34 @@
       <c r="F8" s="3" t="s">
         <v>30</v>
       </c>
-    </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A9" s="1"/>
-      <c r="B9" s="1"/>
-      <c r="C9" s="1"/>
-      <c r="D9" s="1"/>
-      <c r="E9" s="1"/>
-      <c r="F9" s="1"/>
-    </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G8" s="3" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" ht="66" x14ac:dyDescent="0.25">
+      <c r="A9" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="B9" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="C9" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="D9" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="E9" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="F9" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="G9" s="3" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="1"/>
       <c r="B10" s="1"/>
       <c r="C10" s="1"/>
@@ -550,7 +618,7 @@
       <c r="E10" s="1"/>
       <c r="F10" s="1"/>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="1"/>
       <c r="B11" s="1"/>
       <c r="C11" s="1"/>
@@ -558,7 +626,7 @@
       <c r="E11" s="1"/>
       <c r="F11" s="1"/>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="1"/>
       <c r="B12" s="1"/>
       <c r="C12" s="1"/>
@@ -566,7 +634,7 @@
       <c r="E12" s="1"/>
       <c r="F12" s="1"/>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="1"/>
       <c r="B13" s="1"/>
       <c r="C13" s="1"/>
@@ -574,7 +642,7 @@
       <c r="E13" s="1"/>
       <c r="F13" s="1"/>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" s="1"/>
       <c r="B14" s="1"/>
       <c r="C14" s="1"/>
@@ -582,7 +650,7 @@
       <c r="E14" s="1"/>
       <c r="F14" s="1"/>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15" s="1"/>
       <c r="B15" s="1"/>
       <c r="C15" s="1"/>
@@ -590,7 +658,7 @@
       <c r="E15" s="1"/>
       <c r="F15" s="1"/>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" s="1"/>
       <c r="B16" s="1"/>
       <c r="C16" s="1"/>

</xml_diff>